<commit_message>
V2.10 | 08.05.2023 -CICD- 08/05/2023 2:47:23 PM
</commit_message>
<xml_diff>
--- a/Carga Masiva/CargaMaterialesAcrux.xlsx
+++ b/Carga Masiva/CargaMaterialesAcrux.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26529"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RepositoriosAEC\Acrux-Release\Carga Masiva\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED7FA1DA-CD53-4A21-8144-D2715DC9B6C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCB4C9A4-BA92-4AA4-ACAE-15E9A09F3DD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CargaMaterialesAcrux" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
   <si>
     <t>TIPO INVENTARIO</t>
   </si>
@@ -164,6 +164,9 @@
   </si>
   <si>
     <t>UBICACION</t>
+  </si>
+  <si>
+    <t>0-0-0</t>
   </si>
 </sst>
 </file>
@@ -1211,6 +1214,15 @@
       <c r="AA2" t="s">
         <v>42</v>
       </c>
+      <c r="AB2">
+        <v>1</v>
+      </c>
+      <c r="AC2">
+        <v>1</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>48</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>